<commit_message>
Update source layout checks and Sayax tariff output
</commit_message>
<xml_diff>
--- a/06-Haziran/SKF Başlıkları.xlsx
+++ b/06-Haziran/SKF Başlıkları.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\ckvfilesrv01\CLK_ENERJI\Portföy_Yonetimi\Ticari Satış ve Fiyatlama\CK Enerji Ortaklığı - ENO\Gelen Faturalar\Dağıtım Sistem Kullanım Faturaları\2026\SKF Python\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\smocan\Desktop\SKF\06-Haziran\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABE38371-1F9E-4B98-A72D-6F3E3D192CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89E9FF3-1567-4CD8-9475-6939B829CBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="2" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="1" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Başlıklar" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1712" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1755" uniqueCount="527">
   <si>
     <t>Dağıtım Bölgesi</t>
   </si>
@@ -1589,6 +1589,42 @@
   </si>
   <si>
     <t>Sakarya EDAŞ için Aktif Enerji Tüketim (kWh)'ın kaynak dosyadaki Dağıtım Miktarı başlığından etso bazlı olacak şekilde getir (Sütun: AR). Başka bir sütunla herhangi bir işlem yapma.</t>
+  </si>
+  <si>
+    <t>Ticarethaneler</t>
+  </si>
+  <si>
+    <t>Sayax'a Atılacak Tarife</t>
+  </si>
+  <si>
+    <t>Ticarethane TT OG</t>
+  </si>
+  <si>
+    <t>Sanayi TT OG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mesken </t>
+  </si>
+  <si>
+    <t>Mesken TT OG</t>
+  </si>
+  <si>
+    <t>Ticarethane AG</t>
+  </si>
+  <si>
+    <t>Sanayi AG</t>
+  </si>
+  <si>
+    <t>Mesken AG</t>
+  </si>
+  <si>
+    <t>Ticarethane ÇT</t>
+  </si>
+  <si>
+    <t>Sanayi ÇT</t>
+  </si>
+  <si>
+    <t>Mesken ÇT</t>
   </si>
 </sst>
 </file>
@@ -2445,7 +2481,7 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2654,11 +2690,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="45">
@@ -7363,7 +7405,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6115A3-BCAD-4628-8744-E0C82533D896}">
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr defaultColWidth="2.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.77734375" style="37" bestFit="1" customWidth="1"/>
@@ -7374,28 +7416,38 @@
     <col min="6" max="6" width="15.109375" style="37" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.109375" style="37" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.21875" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="2.6640625" style="37"/>
+    <col min="9" max="9" width="12" style="37" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7" style="37" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="37" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" style="37" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="2.6640625" style="37"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70" t="s">
+      <c r="B1" s="71"/>
+      <c r="C1" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70" t="s">
+      <c r="D1" s="71"/>
+      <c r="E1" s="71" t="s">
         <v>218</v>
       </c>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70" t="s">
+      <c r="F1" s="71"/>
+      <c r="G1" s="71" t="s">
         <v>435</v>
       </c>
-      <c r="H1" s="70"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H1" s="71"/>
+      <c r="I1" s="71" t="s">
+        <v>516</v>
+      </c>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="38" t="s">
         <v>337</v>
       </c>
@@ -7420,8 +7472,20 @@
       <c r="H2" s="38" t="s">
         <v>454</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I2" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="38" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="38" t="s">
+        <v>218</v>
+      </c>
+      <c r="L2" s="38" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="37" t="s">
         <v>338</v>
       </c>
@@ -7446,8 +7510,20 @@
       <c r="H3" s="37" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I3" s="73" t="s">
+        <v>385</v>
+      </c>
+      <c r="J3" s="72" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="72" t="s">
+        <v>366</v>
+      </c>
+      <c r="L3" s="72" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="37" t="s">
         <v>343</v>
       </c>
@@ -7472,8 +7548,20 @@
       <c r="H4" s="44" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" s="72" t="s">
+        <v>347</v>
+      </c>
+      <c r="J4" s="72" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="72" t="s">
+        <v>366</v>
+      </c>
+      <c r="L4" s="72" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="37" t="s">
         <v>346</v>
       </c>
@@ -7498,8 +7586,20 @@
       <c r="H5" s="44" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I5" s="72" t="s">
+        <v>519</v>
+      </c>
+      <c r="J5" s="72" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="72" t="s">
+        <v>366</v>
+      </c>
+      <c r="L5" s="72" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>350</v>
       </c>
@@ -7524,8 +7624,20 @@
       <c r="H6" s="44" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6" s="37" t="s">
+        <v>385</v>
+      </c>
+      <c r="J6" s="72" t="s">
+        <v>284</v>
+      </c>
+      <c r="K6" s="72" t="s">
+        <v>366</v>
+      </c>
+      <c r="L6" s="72" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="37" t="s">
         <v>353</v>
       </c>
@@ -7550,8 +7662,20 @@
       <c r="H7" s="45" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7" s="37" t="s">
+        <v>347</v>
+      </c>
+      <c r="J7" s="72" t="s">
+        <v>284</v>
+      </c>
+      <c r="K7" s="72" t="s">
+        <v>366</v>
+      </c>
+      <c r="L7" s="72" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="37" t="s">
         <v>356</v>
       </c>
@@ -7576,8 +7700,20 @@
       <c r="H8" s="44" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8" s="37" t="s">
+        <v>519</v>
+      </c>
+      <c r="J8" s="72" t="s">
+        <v>284</v>
+      </c>
+      <c r="K8" s="72" t="s">
+        <v>366</v>
+      </c>
+      <c r="L8" s="72" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="37" t="s">
         <v>358</v>
       </c>
@@ -7602,8 +7738,20 @@
       <c r="H9" s="37" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9" s="37" t="s">
+        <v>385</v>
+      </c>
+      <c r="J9" s="72" t="s">
+        <v>284</v>
+      </c>
+      <c r="K9" s="72" t="s">
+        <v>342</v>
+      </c>
+      <c r="L9" s="72" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="37" t="s">
         <v>361</v>
       </c>
@@ -7628,8 +7776,20 @@
       <c r="H10" s="37" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10" s="37" t="s">
+        <v>347</v>
+      </c>
+      <c r="J10" s="72" t="s">
+        <v>284</v>
+      </c>
+      <c r="K10" s="72" t="s">
+        <v>342</v>
+      </c>
+      <c r="L10" s="72" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="37" t="s">
         <v>364</v>
       </c>
@@ -7654,8 +7814,20 @@
       <c r="H11" s="37" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11" s="37" t="s">
+        <v>519</v>
+      </c>
+      <c r="J11" s="72" t="s">
+        <v>284</v>
+      </c>
+      <c r="K11" s="72" t="s">
+        <v>342</v>
+      </c>
+      <c r="L11" s="72" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="37" t="s">
         <v>367</v>
       </c>
@@ -7681,7 +7853,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="37" t="s">
         <v>369</v>
       </c>
@@ -7707,7 +7879,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="37" t="s">
         <v>371</v>
       </c>
@@ -7733,7 +7905,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="37" t="s">
         <v>373</v>
       </c>
@@ -7759,7 +7931,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="37" t="s">
         <v>375</v>
       </c>
@@ -8318,6 +8490,12 @@
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="37" t="s">
+        <v>515</v>
+      </c>
+      <c r="B46" s="37" t="s">
+        <v>385</v>
+      </c>
       <c r="G46" s="44" t="s">
         <v>468</v>
       </c>
@@ -8489,11 +8667,12 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G4:H61">
     <sortCondition ref="H3:H61"/>
   </sortState>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="G1:H1"/>
+    <mergeCell ref="I1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9069,7 +9248,7 @@
       <c r="A86" s="42">
         <v>1</v>
       </c>
-      <c r="B86" s="71" t="s">
+      <c r="B86" s="70" t="s">
         <v>514</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Sayax OG tariff corrections
</commit_message>
<xml_diff>
--- a/06-Haziran/SKF Başlıkları.xlsx
+++ b/06-Haziran/SKF Başlıkları.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\smocan\Desktop\SKF\06-Haziran\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89E9FF3-1567-4CD8-9475-6939B829CBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E96140A1-0CBB-48D7-9F59-20E5C9F5AE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="1" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
   </bookViews>
@@ -2693,14 +2693,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="45">
@@ -7424,28 +7424,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71" t="s">
+      <c r="B1" s="73"/>
+      <c r="C1" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71" t="s">
+      <c r="D1" s="73"/>
+      <c r="E1" s="73" t="s">
         <v>218</v>
       </c>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71" t="s">
+      <c r="F1" s="73"/>
+      <c r="G1" s="73" t="s">
         <v>435</v>
       </c>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71" t="s">
+      <c r="H1" s="73"/>
+      <c r="I1" s="73" t="s">
         <v>516</v>
       </c>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="38" t="s">
@@ -7510,16 +7510,16 @@
       <c r="H3" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="73" t="s">
+      <c r="I3" s="72" t="s">
         <v>385</v>
       </c>
-      <c r="J3" s="72" t="s">
+      <c r="J3" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="72" t="s">
+      <c r="K3" s="71" t="s">
         <v>366</v>
       </c>
-      <c r="L3" s="72" t="s">
+      <c r="L3" s="71" t="s">
         <v>517</v>
       </c>
     </row>
@@ -7548,16 +7548,16 @@
       <c r="H4" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="71" t="s">
         <v>347</v>
       </c>
-      <c r="J4" s="72" t="s">
+      <c r="J4" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="K4" s="72" t="s">
+      <c r="K4" s="71" t="s">
         <v>366</v>
       </c>
-      <c r="L4" s="72" t="s">
+      <c r="L4" s="71" t="s">
         <v>518</v>
       </c>
     </row>
@@ -7586,16 +7586,16 @@
       <c r="H5" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="72" t="s">
+      <c r="I5" s="71" t="s">
         <v>519</v>
       </c>
-      <c r="J5" s="72" t="s">
+      <c r="J5" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="72" t="s">
+      <c r="K5" s="71" t="s">
         <v>366</v>
       </c>
-      <c r="L5" s="72" t="s">
+      <c r="L5" s="71" t="s">
         <v>520</v>
       </c>
     </row>
@@ -7627,13 +7627,13 @@
       <c r="I6" s="37" t="s">
         <v>385</v>
       </c>
-      <c r="J6" s="72" t="s">
+      <c r="J6" s="71" t="s">
         <v>284</v>
       </c>
-      <c r="K6" s="72" t="s">
+      <c r="K6" s="71" t="s">
         <v>366</v>
       </c>
-      <c r="L6" s="72" t="s">
+      <c r="L6" s="71" t="s">
         <v>521</v>
       </c>
     </row>
@@ -7665,13 +7665,13 @@
       <c r="I7" s="37" t="s">
         <v>347</v>
       </c>
-      <c r="J7" s="72" t="s">
+      <c r="J7" s="71" t="s">
         <v>284</v>
       </c>
-      <c r="K7" s="72" t="s">
+      <c r="K7" s="71" t="s">
         <v>366</v>
       </c>
-      <c r="L7" s="72" t="s">
+      <c r="L7" s="71" t="s">
         <v>522</v>
       </c>
     </row>
@@ -7703,13 +7703,13 @@
       <c r="I8" s="37" t="s">
         <v>519</v>
       </c>
-      <c r="J8" s="72" t="s">
+      <c r="J8" s="71" t="s">
         <v>284</v>
       </c>
-      <c r="K8" s="72" t="s">
+      <c r="K8" s="71" t="s">
         <v>366</v>
       </c>
-      <c r="L8" s="72" t="s">
+      <c r="L8" s="71" t="s">
         <v>523</v>
       </c>
     </row>
@@ -7741,13 +7741,13 @@
       <c r="I9" s="37" t="s">
         <v>385</v>
       </c>
-      <c r="J9" s="72" t="s">
-        <v>284</v>
-      </c>
-      <c r="K9" s="72" t="s">
+      <c r="J9" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="71" t="s">
         <v>342</v>
       </c>
-      <c r="L9" s="72" t="s">
+      <c r="L9" s="71" t="s">
         <v>524</v>
       </c>
     </row>
@@ -7779,13 +7779,13 @@
       <c r="I10" s="37" t="s">
         <v>347</v>
       </c>
-      <c r="J10" s="72" t="s">
-        <v>284</v>
-      </c>
-      <c r="K10" s="72" t="s">
+      <c r="J10" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="71" t="s">
         <v>342</v>
       </c>
-      <c r="L10" s="72" t="s">
+      <c r="L10" s="71" t="s">
         <v>525</v>
       </c>
     </row>
@@ -7817,13 +7817,13 @@
       <c r="I11" s="37" t="s">
         <v>519</v>
       </c>
-      <c r="J11" s="72" t="s">
-        <v>284</v>
-      </c>
-      <c r="K11" s="72" t="s">
+      <c r="J11" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="K11" s="71" t="s">
         <v>342</v>
       </c>
-      <c r="L11" s="72" t="s">
+      <c r="L11" s="71" t="s">
         <v>526</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SenaV3: save current SKF download output
</commit_message>
<xml_diff>
--- a/06-Haziran/SKF Başlıkları.xlsx
+++ b/06-Haziran/SKF Başlıkları.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\smocan\Desktop\SKF\06-Haziran\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E96140A1-0CBB-48D7-9F59-20E5C9F5AE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB9B65A-8AA6-4FFE-818B-B7ADD624C2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="1" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="4" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Başlıklar" sheetId="1" r:id="rId1"/>
     <sheet name="Düzeltme" sheetId="9" r:id="rId2"/>
     <sheet name="Notlar" sheetId="2" r:id="rId3"/>
+    <sheet name="Tarifeler" sheetId="10" r:id="rId4"/>
+    <sheet name="Bizim Kestiğimiz 2" sheetId="11" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Başlıklar!$A$1:$AG$23</definedName>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1755" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1884" uniqueCount="555">
   <si>
     <t>Dağıtım Bölgesi</t>
   </si>
@@ -1625,6 +1627,92 @@
   </si>
   <si>
     <t>Mesken ÇT</t>
+  </si>
+  <si>
+    <t>İSK Sanayi</t>
+  </si>
+  <si>
+    <t>DSK Ticarethane TT AG</t>
+  </si>
+  <si>
+    <t>DSK Ticarethane TT OG</t>
+  </si>
+  <si>
+    <t>DSK Ticarethane ÇT OG</t>
+  </si>
+  <si>
+    <t>DSK Sanayi TT OG</t>
+  </si>
+  <si>
+    <t>DSK Sanayi TT AG</t>
+  </si>
+  <si>
+    <t>DSK Sanayi ÇT OG</t>
+  </si>
+  <si>
+    <t>DSK Mesken TT OG</t>
+  </si>
+  <si>
+    <t>DSK Mesken TT AG</t>
+  </si>
+  <si>
+    <t>DSK Mesken ÇT OG</t>
+  </si>
+  <si>
+    <t>OG Çift Terim</t>
+  </si>
+  <si>
+    <t>Dağıtım Bedeli
+(kr/kWh)</t>
+  </si>
+  <si>
+    <t>Kamu ve Özel Hizmetler Sektörü ile Diğer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dağıtım Sistemi Kullanıcıları </t>
+  </si>
+  <si>
+    <t>Abone / Kullanıcı Grubu</t>
+  </si>
+  <si>
+    <t>Dağıtım Sistemi Kullanıcısı Üretici ve Tüketiciler İçin Dağıtım Sistem Kullanım Bedelleri</t>
+  </si>
+  <si>
+    <t>OG Tek Terim</t>
+  </si>
+  <si>
+    <t>İletim Sistemi Kullanıcıları</t>
+  </si>
+  <si>
+    <t>AG Tek Terim</t>
+  </si>
+  <si>
+    <t>Satır</t>
+  </si>
+  <si>
+    <t>Terim Tipi</t>
+  </si>
+  <si>
+    <t>Güç kW</t>
+  </si>
+  <si>
+    <t>Güç Bedeli(TL)</t>
+  </si>
+  <si>
+    <t>Reaktif Bedel (TL)</t>
+  </si>
+  <si>
+    <t>Olması Gereken Dağıtım Bedeli (TL)</t>
+  </si>
+  <si>
+    <t>Açılacak Başlık</t>
+  </si>
+  <si>
+    <t>Alınacak Sütun</t>
+  </si>
+  <si>
+    <t>Güç Bedeli
+(kr/kW/ay)</t>
   </si>
 </sst>
 </file>
@@ -1634,7 +1722,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1916,8 +2004,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8.25"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2138,8 +2240,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -2433,8 +2540,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="45">
+  <cellStyleXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2480,8 +2611,9 @@
     <xf numFmtId="0" fontId="11" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2699,11 +2831,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="36" fillId="40" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="37" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="37" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="43" fontId="37" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="45">
+  <cellStyles count="46">
     <cellStyle name="%20 - Vurgu1" xfId="20" builtinId="30" customBuiltin="1"/>
     <cellStyle name="%20 - Vurgu2" xfId="24" builtinId="34" customBuiltin="1"/>
     <cellStyle name="%20 - Vurgu3" xfId="28" builtinId="38" customBuiltin="1"/>
@@ -2738,6 +2893,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="43" xr:uid="{C509D5A2-FA51-4001-B741-553F48808D92}"/>
     <cellStyle name="Normal 3" xfId="44" xr:uid="{81023F4B-1BC7-425F-A8CF-0DDD0B8AE1FA}"/>
+    <cellStyle name="Normal 646" xfId="45" xr:uid="{D9207873-F055-42AB-8BA9-D5B5125AE9DF}"/>
     <cellStyle name="Not" xfId="16" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Nötr" xfId="9" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Toplam" xfId="18" builtinId="25" customBuiltin="1"/>
@@ -7424,28 +7580,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73" t="s">
+      <c r="B1" s="74"/>
+      <c r="C1" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73" t="s">
+      <c r="D1" s="74"/>
+      <c r="E1" s="74" t="s">
         <v>218</v>
       </c>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73" t="s">
+      <c r="F1" s="74"/>
+      <c r="G1" s="74" t="s">
         <v>435</v>
       </c>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73" t="s">
+      <c r="H1" s="74"/>
+      <c r="I1" s="74" t="s">
         <v>516</v>
       </c>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="38" t="s">
@@ -9272,4 +9428,555 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA00C5E4-961E-42C0-B3EE-89E924EDC3DF}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="42.109375" customWidth="1"/>
+    <col min="4" max="4" width="69.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="73" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C1" t="s">
+        <v>541</v>
+      </c>
+      <c r="D1" t="s">
+        <v>542</v>
+      </c>
+      <c r="E1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>527</v>
+      </c>
+      <c r="C2" t="s">
+        <v>544</v>
+      </c>
+      <c r="D2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>528</v>
+      </c>
+      <c r="B3" t="s">
+        <v>545</v>
+      </c>
+      <c r="C3" t="s">
+        <v>539</v>
+      </c>
+      <c r="D3" t="s">
+        <v>538</v>
+      </c>
+      <c r="E3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B4" t="s">
+        <v>543</v>
+      </c>
+      <c r="C4" t="s">
+        <v>539</v>
+      </c>
+      <c r="D4" t="s">
+        <v>538</v>
+      </c>
+      <c r="E4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>530</v>
+      </c>
+      <c r="B5" t="s">
+        <v>537</v>
+      </c>
+      <c r="C5" t="s">
+        <v>539</v>
+      </c>
+      <c r="D5" t="s">
+        <v>538</v>
+      </c>
+      <c r="E5" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>531</v>
+      </c>
+      <c r="B6" t="s">
+        <v>543</v>
+      </c>
+      <c r="C6" t="s">
+        <v>347</v>
+      </c>
+      <c r="D6" t="s">
+        <v>538</v>
+      </c>
+      <c r="E6" t="s">
+        <v>171</v>
+      </c>
+      <c r="F6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>532</v>
+      </c>
+      <c r="B7" t="s">
+        <v>545</v>
+      </c>
+      <c r="C7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D7" t="s">
+        <v>538</v>
+      </c>
+      <c r="E7" t="s">
+        <v>171</v>
+      </c>
+      <c r="F7">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>533</v>
+      </c>
+      <c r="B8" t="s">
+        <v>537</v>
+      </c>
+      <c r="C8" t="s">
+        <v>347</v>
+      </c>
+      <c r="D8" t="s">
+        <v>538</v>
+      </c>
+      <c r="E8" t="s">
+        <v>171</v>
+      </c>
+      <c r="F8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>534</v>
+      </c>
+      <c r="B9" t="s">
+        <v>543</v>
+      </c>
+      <c r="C9" t="s">
+        <v>339</v>
+      </c>
+      <c r="D9" t="s">
+        <v>538</v>
+      </c>
+      <c r="E9" t="s">
+        <v>171</v>
+      </c>
+      <c r="F9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>535</v>
+      </c>
+      <c r="B10" t="s">
+        <v>545</v>
+      </c>
+      <c r="C10" t="s">
+        <v>339</v>
+      </c>
+      <c r="D10" t="s">
+        <v>538</v>
+      </c>
+      <c r="E10" t="s">
+        <v>171</v>
+      </c>
+      <c r="F10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>536</v>
+      </c>
+      <c r="B11" t="s">
+        <v>537</v>
+      </c>
+      <c r="C11" t="s">
+        <v>339</v>
+      </c>
+      <c r="D11" t="s">
+        <v>538</v>
+      </c>
+      <c r="E11" t="s">
+        <v>171</v>
+      </c>
+      <c r="F11">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2B99A2-E2AD-46AF-8B85-282DC4420555}">
+  <dimension ref="A1:N28"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="36" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>552</v>
+      </c>
+      <c r="B1" s="75" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="75" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="75" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="75" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="75" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="75" t="s">
+        <v>547</v>
+      </c>
+      <c r="H1" s="75" t="s">
+        <v>217</v>
+      </c>
+      <c r="I1" s="76" t="s">
+        <v>548</v>
+      </c>
+      <c r="J1" s="76" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="76" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="76" t="s">
+        <v>549</v>
+      </c>
+      <c r="M1" s="76" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="76" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="48" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>553</v>
+      </c>
+      <c r="B2" s="75" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="75" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="75" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="75" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="75" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="76" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="77" t="s">
+        <v>551</v>
+      </c>
+      <c r="L2" s="76" t="s">
+        <v>549</v>
+      </c>
+      <c r="M2" s="76" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" s="76" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B5" s="79" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="79" t="s">
+        <v>547</v>
+      </c>
+      <c r="D5" s="79" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B6" s="78" t="s">
+        <v>527</v>
+      </c>
+      <c r="C6" s="78"/>
+      <c r="D6" s="78"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B7" s="78" t="s">
+        <v>528</v>
+      </c>
+      <c r="C7" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="D7" s="78" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B8" s="78" t="s">
+        <v>529</v>
+      </c>
+      <c r="C8" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="D8" s="78" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B9" s="78" t="s">
+        <v>530</v>
+      </c>
+      <c r="C9" s="78" t="s">
+        <v>342</v>
+      </c>
+      <c r="D9" s="78" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B10" s="78" t="s">
+        <v>531</v>
+      </c>
+      <c r="C10" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="D10" s="78" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B11" s="78" t="s">
+        <v>532</v>
+      </c>
+      <c r="C11" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="D11" s="78" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B12" s="78" t="s">
+        <v>533</v>
+      </c>
+      <c r="C12" s="78" t="s">
+        <v>342</v>
+      </c>
+      <c r="D12" s="78" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B13" s="78" t="s">
+        <v>534</v>
+      </c>
+      <c r="C13" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="D13" s="78" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B14" s="78" t="s">
+        <v>535</v>
+      </c>
+      <c r="C14" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="D14" s="78" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B15" s="78" t="s">
+        <v>536</v>
+      </c>
+      <c r="C15" s="78" t="s">
+        <v>342</v>
+      </c>
+      <c r="D15" s="78" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B17" s="82"/>
+      <c r="C17" s="82"/>
+      <c r="D17" s="82"/>
+      <c r="E17" s="82"/>
+      <c r="F17" s="82"/>
+      <c r="G17" s="82"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B18" s="79" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="78" t="s">
+        <v>541</v>
+      </c>
+      <c r="D18" s="78" t="s">
+        <v>542</v>
+      </c>
+      <c r="E18" s="78" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" s="78" t="s">
+        <v>546</v>
+      </c>
+      <c r="G18" s="81" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B19" s="78" t="s">
+        <v>347</v>
+      </c>
+      <c r="C19" s="78" t="s">
+        <v>347</v>
+      </c>
+      <c r="D19" s="78" t="s">
+        <v>554</v>
+      </c>
+      <c r="E19" s="78" t="s">
+        <v>168</v>
+      </c>
+      <c r="F19" s="78">
+        <v>7</v>
+      </c>
+      <c r="G19" s="81"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="78" t="s">
+        <v>385</v>
+      </c>
+      <c r="C20" s="78" t="s">
+        <v>539</v>
+      </c>
+      <c r="D20" s="78" t="s">
+        <v>554</v>
+      </c>
+      <c r="E20" s="78" t="s">
+        <v>168</v>
+      </c>
+      <c r="F20" s="78">
+        <v>8</v>
+      </c>
+      <c r="G20" s="78"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B21" s="78" t="s">
+        <v>339</v>
+      </c>
+      <c r="C21" s="78" t="s">
+        <v>339</v>
+      </c>
+      <c r="D21" s="78" t="s">
+        <v>554</v>
+      </c>
+      <c r="E21" s="78" t="s">
+        <v>168</v>
+      </c>
+      <c r="F21" s="78">
+        <v>9</v>
+      </c>
+      <c r="G21" s="78"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B22" s="80"/>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="80"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B24" s="80"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B25" s="80"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B26" s="80"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B27" s="80"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B28" s="80"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B17:G17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add region invoice summaries and reconciliation consumption reports
</commit_message>
<xml_diff>
--- a/06-Haziran/SKF Başlıkları.xlsx
+++ b/06-Haziran/SKF Başlıkları.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\smocan\Desktop\SKF\06-Haziran\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB9B65A-8AA6-4FFE-818B-B7ADD624C2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC32C47-7F09-46EA-9FE6-0E3867D371C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="4" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="738" activeTab="5" xr2:uid="{BA6614F6-086B-4C10-AE8B-B1AF864793CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Başlıklar" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Notlar" sheetId="2" r:id="rId3"/>
     <sheet name="Tarifeler" sheetId="10" r:id="rId4"/>
     <sheet name="Bizim Kestiğimiz 2" sheetId="11" r:id="rId5"/>
+    <sheet name="Bölge Bizim Kestiğmiz" sheetId="12" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Başlıklar!$A$1:$AG$23</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1884" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1969" uniqueCount="581">
   <si>
     <t>Dağıtım Bölgesi</t>
   </si>
@@ -1713,6 +1714,84 @@
   <si>
     <t>Güç Bedeli
 (kr/kW/ay)</t>
+  </si>
+  <si>
+    <t>Aktik Kayıp</t>
+  </si>
+  <si>
+    <t>AG-OG</t>
+  </si>
+  <si>
+    <t>AG/OG</t>
+  </si>
+  <si>
+    <t>CW</t>
+  </si>
+  <si>
+    <t>Fatura Abone Grubu2</t>
+  </si>
+  <si>
+    <t>Aktif Enerji (kwh)</t>
+  </si>
+  <si>
+    <t>Toplam Dağıtım Bedeli</t>
+  </si>
+  <si>
+    <t>BU</t>
+  </si>
+  <si>
+    <t>Güç aşım Bedeli</t>
+  </si>
+  <si>
+    <t>Reaktif Bedel + Enerji Bedeli Net Reaktif İhlal</t>
+  </si>
+  <si>
+    <t>Kamu/Özel Sektör ve Diğer</t>
+  </si>
+  <si>
+    <t>Düzeltme</t>
+  </si>
+  <si>
+    <t>Yükelenen</t>
+  </si>
+  <si>
+    <t>Başlık</t>
+  </si>
+  <si>
+    <t>Bizim Kestiğimiz 2'ye Alırken Düzeltme</t>
+  </si>
+  <si>
+    <t>Kdv</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>KDV Matrahı</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>TOPLAM</t>
+  </si>
+  <si>
+    <t>Fatura Tutarı</t>
+  </si>
+  <si>
+    <t>Aktif Enerji TL</t>
+  </si>
+  <si>
+    <t>Toplam enerji Bedeli(Aktif+Trafo Kaybı+Ek Tüketim+PSH)</t>
+  </si>
+  <si>
+    <t>Btv Bedeli</t>
+  </si>
+  <si>
+    <t>BTV</t>
+  </si>
+  <si>
+    <t>Fiyat Farkı</t>
   </si>
 </sst>
 </file>
@@ -1722,7 +1801,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="39" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2008,10 +2087,21 @@
       <sz val="8.25"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="162"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -2613,7 +2703,7 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2712,9 +2802,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2834,9 +2921,6 @@
     <xf numFmtId="49" fontId="36" fillId="40" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="37" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2854,7 +2938,17 @@
     <xf numFmtId="43" fontId="37" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3781,22 +3875,22 @@
       <c r="AC2" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="AD2" s="58" t="s">
+      <c r="AD2" s="57" t="s">
         <v>106</v>
       </c>
-      <c r="AE2" s="59" t="s">
+      <c r="AE2" s="58" t="s">
         <v>163</v>
       </c>
-      <c r="AF2" s="60" t="s">
+      <c r="AF2" s="59" t="s">
         <v>105</v>
       </c>
       <c r="AG2" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="AH2" s="50" t="s">
+      <c r="AH2" s="49" t="s">
         <v>285</v>
       </c>
-      <c r="AI2" s="36" t="s">
+      <c r="AI2" s="35" t="s">
         <v>202</v>
       </c>
       <c r="AJ2" s="16" t="s">
@@ -3811,58 +3905,58 @@
       <c r="AM2" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN2" s="50" t="s">
+      <c r="AN2" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="AO2" s="36" t="s">
+      <c r="AO2" s="35" t="s">
         <v>299</v>
       </c>
-      <c r="AP2" s="50" t="s">
+      <c r="AP2" s="49" t="s">
         <v>300</v>
       </c>
-      <c r="AQ2" s="36" t="s">
+      <c r="AQ2" s="35" t="s">
         <v>201</v>
       </c>
-      <c r="AR2" s="50" t="s">
+      <c r="AR2" s="49" t="s">
         <v>301</v>
       </c>
-      <c r="AS2" s="36" t="s">
+      <c r="AS2" s="35" t="s">
         <v>174</v>
       </c>
-      <c r="AT2" s="50" t="s">
+      <c r="AT2" s="49" t="s">
         <v>302</v>
       </c>
-      <c r="AU2" s="36" t="s">
+      <c r="AU2" s="35" t="s">
         <v>195</v>
       </c>
-      <c r="AV2" s="51" t="s">
+      <c r="AV2" s="50" t="s">
         <v>303</v>
       </c>
-      <c r="AW2" s="36" t="s">
+      <c r="AW2" s="35" t="s">
         <v>304</v>
       </c>
-      <c r="AX2" s="50" t="s">
+      <c r="AX2" s="49" t="s">
         <v>305</v>
       </c>
-      <c r="AY2" s="36" t="s">
+      <c r="AY2" s="35" t="s">
         <v>306</v>
       </c>
-      <c r="AZ2" s="50" t="s">
+      <c r="AZ2" s="49" t="s">
         <v>307</v>
       </c>
-      <c r="BA2" s="36" t="s">
+      <c r="BA2" s="35" t="s">
         <v>220</v>
       </c>
-      <c r="BB2" s="50" t="s">
+      <c r="BB2" s="49" t="s">
         <v>308</v>
       </c>
-      <c r="BC2" s="36" t="s">
+      <c r="BC2" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="BD2" s="50" t="s">
+      <c r="BD2" s="49" t="s">
         <v>309</v>
       </c>
-      <c r="BE2" s="36" t="s">
+      <c r="BE2" s="35" t="s">
         <v>310</v>
       </c>
     </row>
@@ -3984,7 +4078,7 @@
       <c r="AM3" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN3" s="36" t="s">
+      <c r="AN3" s="35" t="s">
         <v>311</v>
       </c>
       <c r="AO3" s="16" t="s">
@@ -4139,10 +4233,10 @@
       <c r="AG4" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="49" t="s">
         <v>285</v>
       </c>
-      <c r="AI4" s="36" t="s">
+      <c r="AI4" s="35" t="s">
         <v>195</v>
       </c>
       <c r="AJ4" s="16" t="s">
@@ -4255,7 +4349,7 @@
       <c r="N5" s="16" t="s">
         <v>510</v>
       </c>
-      <c r="O5" s="68" t="s">
+      <c r="O5" s="67" t="s">
         <v>187</v>
       </c>
       <c r="P5" s="9" t="s">
@@ -4312,10 +4406,10 @@
       <c r="AG5" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH5" s="52" t="s">
+      <c r="AH5" s="51" t="s">
         <v>286</v>
       </c>
-      <c r="AI5" s="36" t="s">
+      <c r="AI5" s="35" t="s">
         <v>173</v>
       </c>
       <c r="AJ5" s="16" t="s">
@@ -4330,10 +4424,10 @@
       <c r="AM5" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN5" s="52" t="s">
+      <c r="AN5" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="AO5" s="36" t="s">
+      <c r="AO5" s="35" t="s">
         <v>226</v>
       </c>
       <c r="AP5" s="16" t="s">
@@ -4849,28 +4943,28 @@
       <c r="AM8" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN8" s="53" t="s">
+      <c r="AN8" s="52" t="s">
         <v>313</v>
       </c>
-      <c r="AO8" s="36" t="s">
+      <c r="AO8" s="35" t="s">
         <v>306</v>
       </c>
-      <c r="AP8" s="53" t="s">
+      <c r="AP8" s="52" t="s">
         <v>314</v>
       </c>
-      <c r="AQ8" s="36" t="s">
+      <c r="AQ8" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="AR8" s="53" t="s">
+      <c r="AR8" s="52" t="s">
         <v>315</v>
       </c>
-      <c r="AS8" s="36" t="s">
+      <c r="AS8" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="AT8" s="53" t="s">
+      <c r="AT8" s="52" t="s">
         <v>316</v>
       </c>
-      <c r="AU8" s="36" t="s">
+      <c r="AU8" s="35" t="s">
         <v>220</v>
       </c>
       <c r="AV8" s="16" t="s">
@@ -4911,7 +5005,7 @@
       <c r="B9" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="69" t="s">
+      <c r="C9" s="68" t="s">
         <v>176</v>
       </c>
       <c r="D9" s="28" t="s">
@@ -4923,19 +5017,19 @@
       <c r="F9" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="69" t="s">
+      <c r="G9" s="68" t="s">
         <v>180</v>
       </c>
       <c r="H9" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="69" t="s">
+      <c r="I9" s="68" t="s">
         <v>180</v>
       </c>
       <c r="J9" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="69" t="s">
+      <c r="K9" s="68" t="s">
         <v>180</v>
       </c>
       <c r="L9" s="16" t="s">
@@ -5022,10 +5116,10 @@
       <c r="AM9" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN9" s="54" t="s">
+      <c r="AN9" s="53" t="s">
         <v>317</v>
       </c>
-      <c r="AO9" s="36" t="s">
+      <c r="AO9" s="35" t="s">
         <v>188</v>
       </c>
       <c r="AP9" s="16" t="s">
@@ -5120,7 +5214,7 @@
       <c r="N10" s="16" t="s">
         <v>510</v>
       </c>
-      <c r="O10" s="68" t="s">
+      <c r="O10" s="67" t="s">
         <v>187</v>
       </c>
       <c r="P10" s="9" t="s">
@@ -5177,10 +5271,10 @@
       <c r="AG10" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH10" s="52" t="s">
+      <c r="AH10" s="51" t="s">
         <v>286</v>
       </c>
-      <c r="AI10" s="36" t="s">
+      <c r="AI10" s="35" t="s">
         <v>173</v>
       </c>
       <c r="AJ10" s="16" t="s">
@@ -5195,10 +5289,10 @@
       <c r="AM10" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN10" s="52" t="s">
+      <c r="AN10" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="AO10" s="36" t="s">
+      <c r="AO10" s="35" t="s">
         <v>226</v>
       </c>
       <c r="AP10" s="16" t="s">
@@ -5427,25 +5521,25 @@
       <c r="A12" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="60" t="s">
         <v>417</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="D12" s="61" t="s">
+      <c r="D12" s="60" t="s">
         <v>37</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>486</v>
       </c>
-      <c r="F12" s="61" t="s">
+      <c r="F12" s="60" t="s">
         <v>485</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="61" t="s">
+      <c r="H12" s="60" t="s">
         <v>487</v>
       </c>
       <c r="I12" s="10" t="s">
@@ -5457,19 +5551,19 @@
       <c r="K12" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="L12" s="61" t="s">
+      <c r="L12" s="60" t="s">
         <v>502</v>
       </c>
       <c r="M12" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="N12" s="61" t="s">
+      <c r="N12" s="60" t="s">
         <v>91</v>
       </c>
-      <c r="O12" s="47" t="s">
+      <c r="O12" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="P12" s="61" t="s">
+      <c r="P12" s="60" t="s">
         <v>501</v>
       </c>
       <c r="Q12" s="10" t="s">
@@ -5481,25 +5575,25 @@
       <c r="S12" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="T12" s="61" t="s">
+      <c r="T12" s="60" t="s">
         <v>14</v>
       </c>
       <c r="U12" s="10" t="s">
         <v>491</v>
       </c>
-      <c r="V12" s="61" t="s">
+      <c r="V12" s="60" t="s">
         <v>12</v>
       </c>
       <c r="W12" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="X12" s="61" t="s">
+      <c r="X12" s="60" t="s">
         <v>13</v>
       </c>
       <c r="Y12" s="10" t="s">
         <v>494</v>
       </c>
-      <c r="Z12" s="61" t="s">
+      <c r="Z12" s="60" t="s">
         <v>489</v>
       </c>
       <c r="AA12" s="10" t="s">
@@ -5511,10 +5605,10 @@
       <c r="AC12" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AD12" s="61" t="s">
+      <c r="AD12" s="60" t="s">
         <v>503</v>
       </c>
-      <c r="AE12" s="48" t="s">
+      <c r="AE12" s="47" t="s">
         <v>504</v>
       </c>
       <c r="AF12" s="16" t="s">
@@ -5523,10 +5617,10 @@
       <c r="AG12" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH12" s="61" t="s">
+      <c r="AH12" s="60" t="s">
         <v>492</v>
       </c>
-      <c r="AI12" s="47" t="s">
+      <c r="AI12" s="46" t="s">
         <v>493</v>
       </c>
       <c r="AJ12" s="16" t="s">
@@ -5541,28 +5635,28 @@
       <c r="AM12" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN12" s="61" t="s">
+      <c r="AN12" s="60" t="s">
         <v>495</v>
       </c>
-      <c r="AO12" s="47" t="s">
+      <c r="AO12" s="46" t="s">
         <v>496</v>
       </c>
-      <c r="AP12" s="61" t="s">
+      <c r="AP12" s="60" t="s">
         <v>329</v>
       </c>
-      <c r="AQ12" s="47" t="s">
+      <c r="AQ12" s="46" t="s">
         <v>497</v>
       </c>
-      <c r="AR12" s="61" t="s">
+      <c r="AR12" s="60" t="s">
         <v>498</v>
       </c>
-      <c r="AS12" s="47" t="s">
+      <c r="AS12" s="46" t="s">
         <v>499</v>
       </c>
-      <c r="AT12" s="61" t="s">
+      <c r="AT12" s="60" t="s">
         <v>500</v>
       </c>
-      <c r="AU12" s="47" t="s">
+      <c r="AU12" s="46" t="s">
         <v>206</v>
       </c>
       <c r="AV12" s="16" t="s">
@@ -5696,10 +5790,10 @@
       <c r="AG13" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH13" s="52" t="s">
+      <c r="AH13" s="51" t="s">
         <v>286</v>
       </c>
-      <c r="AI13" s="36" t="s">
+      <c r="AI13" s="35" t="s">
         <v>173</v>
       </c>
       <c r="AJ13" s="16" t="s">
@@ -5714,10 +5808,10 @@
       <c r="AM13" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN13" s="52" t="s">
+      <c r="AN13" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="AO13" s="36" t="s">
+      <c r="AO13" s="35" t="s">
         <v>226</v>
       </c>
       <c r="AP13" s="16" t="s">
@@ -5857,22 +5951,22 @@
       <c r="AC14" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="AD14" s="58" t="s">
+      <c r="AD14" s="57" t="s">
         <v>106</v>
       </c>
-      <c r="AE14" s="59" t="s">
+      <c r="AE14" s="58" t="s">
         <v>163</v>
       </c>
-      <c r="AF14" s="60" t="s">
+      <c r="AF14" s="59" t="s">
         <v>105</v>
       </c>
       <c r="AG14" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="AH14" s="50" t="s">
+      <c r="AH14" s="49" t="s">
         <v>285</v>
       </c>
-      <c r="AI14" s="36" t="s">
+      <c r="AI14" s="35" t="s">
         <v>202</v>
       </c>
       <c r="AJ14" s="16" t="s">
@@ -5887,58 +5981,58 @@
       <c r="AM14" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN14" s="50" t="s">
+      <c r="AN14" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="AO14" s="36" t="s">
+      <c r="AO14" s="35" t="s">
         <v>299</v>
       </c>
-      <c r="AP14" s="50" t="s">
+      <c r="AP14" s="49" t="s">
         <v>300</v>
       </c>
-      <c r="AQ14" s="36" t="s">
+      <c r="AQ14" s="35" t="s">
         <v>201</v>
       </c>
-      <c r="AR14" s="50" t="s">
+      <c r="AR14" s="49" t="s">
         <v>301</v>
       </c>
-      <c r="AS14" s="36" t="s">
+      <c r="AS14" s="35" t="s">
         <v>174</v>
       </c>
-      <c r="AT14" s="50" t="s">
+      <c r="AT14" s="49" t="s">
         <v>302</v>
       </c>
-      <c r="AU14" s="36" t="s">
+      <c r="AU14" s="35" t="s">
         <v>195</v>
       </c>
-      <c r="AV14" s="51" t="s">
+      <c r="AV14" s="50" t="s">
         <v>303</v>
       </c>
-      <c r="AW14" s="36" t="s">
+      <c r="AW14" s="35" t="s">
         <v>304</v>
       </c>
-      <c r="AX14" s="50" t="s">
+      <c r="AX14" s="49" t="s">
         <v>305</v>
       </c>
-      <c r="AY14" s="36" t="s">
+      <c r="AY14" s="35" t="s">
         <v>306</v>
       </c>
-      <c r="AZ14" s="50" t="s">
+      <c r="AZ14" s="49" t="s">
         <v>307</v>
       </c>
-      <c r="BA14" s="36" t="s">
+      <c r="BA14" s="35" t="s">
         <v>220</v>
       </c>
-      <c r="BB14" s="50" t="s">
+      <c r="BB14" s="49" t="s">
         <v>308</v>
       </c>
-      <c r="BC14" s="36" t="s">
+      <c r="BC14" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="BD14" s="50" t="s">
+      <c r="BD14" s="49" t="s">
         <v>309</v>
       </c>
-      <c r="BE14" s="36" t="s">
+      <c r="BE14" s="35" t="s">
         <v>310</v>
       </c>
     </row>
@@ -6191,7 +6285,7 @@
       <c r="Y16" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="Z16" s="62" t="s">
+      <c r="Z16" s="61" t="s">
         <v>258</v>
       </c>
       <c r="AA16" s="10" t="s">
@@ -6233,34 +6327,34 @@
       <c r="AM16" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN16" s="55" t="s">
+      <c r="AN16" s="54" t="s">
         <v>318</v>
       </c>
-      <c r="AO16" s="36" t="s">
+      <c r="AO16" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="AP16" s="55" t="s">
+      <c r="AP16" s="54" t="s">
         <v>319</v>
       </c>
-      <c r="AQ16" s="36" t="s">
+      <c r="AQ16" s="35" t="s">
         <v>195</v>
       </c>
-      <c r="AR16" s="55" t="s">
+      <c r="AR16" s="54" t="s">
         <v>316</v>
       </c>
-      <c r="AS16" s="36" t="s">
+      <c r="AS16" s="35" t="s">
         <v>304</v>
       </c>
-      <c r="AT16" s="55" t="s">
+      <c r="AT16" s="54" t="s">
         <v>320</v>
       </c>
-      <c r="AU16" s="36" t="s">
+      <c r="AU16" s="35" t="s">
         <v>306</v>
       </c>
-      <c r="AV16" s="55" t="s">
+      <c r="AV16" s="54" t="s">
         <v>321</v>
       </c>
-      <c r="AW16" s="36" t="s">
+      <c r="AW16" s="35" t="s">
         <v>220</v>
       </c>
       <c r="AX16" s="16" t="s">
@@ -6388,7 +6482,7 @@
       <c r="AG17" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH17" s="56" t="s">
+      <c r="AH17" s="55" t="s">
         <v>287</v>
       </c>
       <c r="AI17" s="20" t="s">
@@ -6406,16 +6500,16 @@
       <c r="AM17" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN17" s="56" t="s">
+      <c r="AN17" s="55" t="s">
         <v>322</v>
       </c>
-      <c r="AO17" s="36" t="s">
+      <c r="AO17" s="35" t="s">
         <v>323</v>
       </c>
-      <c r="AP17" s="56" t="s">
+      <c r="AP17" s="55" t="s">
         <v>324</v>
       </c>
-      <c r="AQ17" s="36" t="s">
+      <c r="AQ17" s="35" t="s">
         <v>325</v>
       </c>
       <c r="AR17" s="16" t="s">
@@ -6471,25 +6565,25 @@
       <c r="C18" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" s="62" t="s">
         <v>216</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="F18" s="63" t="s">
+      <c r="F18" s="62" t="s">
         <v>20</v>
       </c>
       <c r="G18" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="H18" s="63" t="s">
+      <c r="H18" s="62" t="s">
         <v>217</v>
       </c>
       <c r="I18" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="J18" s="63" t="s">
+      <c r="J18" s="62" t="s">
         <v>218</v>
       </c>
       <c r="K18" s="17" t="s">
@@ -6501,16 +6595,16 @@
       <c r="M18" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="N18" s="63" t="s">
+      <c r="N18" s="62" t="s">
         <v>91</v>
       </c>
       <c r="O18" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="P18" s="64" t="s">
+      <c r="P18" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="Q18" s="48" t="s">
+      <c r="Q18" s="47" t="s">
         <v>228</v>
       </c>
       <c r="R18" s="16" t="s">
@@ -6519,25 +6613,25 @@
       <c r="S18" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="T18" s="63" t="s">
+      <c r="T18" s="62" t="s">
         <v>14</v>
       </c>
       <c r="U18" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="V18" s="63" t="s">
+      <c r="V18" s="62" t="s">
         <v>222</v>
       </c>
       <c r="W18" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="X18" s="63" t="s">
+      <c r="X18" s="62" t="s">
         <v>13</v>
       </c>
       <c r="Y18" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="Z18" s="63" t="s">
+      <c r="Z18" s="62" t="s">
         <v>223</v>
       </c>
       <c r="AA18" s="17" t="s">
@@ -6549,7 +6643,7 @@
       <c r="AC18" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AD18" s="63" t="s">
+      <c r="AD18" s="62" t="s">
         <v>225</v>
       </c>
       <c r="AE18" s="17" t="s">
@@ -6561,16 +6655,16 @@
       <c r="AG18" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH18" s="50" t="s">
+      <c r="AH18" s="49" t="s">
         <v>285</v>
       </c>
-      <c r="AI18" s="36" t="s">
+      <c r="AI18" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="AJ18" s="50" t="s">
+      <c r="AJ18" s="49" t="s">
         <v>294</v>
       </c>
-      <c r="AK18" s="36" t="s">
+      <c r="AK18" s="35" t="s">
         <v>295</v>
       </c>
       <c r="AL18" s="16" t="s">
@@ -6579,34 +6673,34 @@
       <c r="AM18" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN18" s="50" t="s">
+      <c r="AN18" s="49" t="s">
         <v>303</v>
       </c>
-      <c r="AO18" s="36" t="s">
+      <c r="AO18" s="35" t="s">
         <v>326</v>
       </c>
-      <c r="AP18" s="50" t="s">
+      <c r="AP18" s="49" t="s">
         <v>327</v>
       </c>
-      <c r="AQ18" s="36" t="s">
+      <c r="AQ18" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="AR18" s="50" t="s">
+      <c r="AR18" s="49" t="s">
         <v>328</v>
       </c>
-      <c r="AS18" s="36" t="s">
+      <c r="AS18" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="AT18" s="50" t="s">
+      <c r="AT18" s="49" t="s">
         <v>301</v>
       </c>
-      <c r="AU18" s="36" t="s">
+      <c r="AU18" s="35" t="s">
         <v>290</v>
       </c>
-      <c r="AV18" s="50" t="s">
+      <c r="AV18" s="49" t="s">
         <v>329</v>
       </c>
-      <c r="AW18" s="36" t="s">
+      <c r="AW18" s="35" t="s">
         <v>208</v>
       </c>
       <c r="AX18" s="16" t="s">
@@ -6811,7 +6905,7 @@
       <c r="A20" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="B20" s="63" t="s">
+      <c r="B20" s="62" t="s">
         <v>227</v>
       </c>
       <c r="C20" s="17" t="s">
@@ -6853,16 +6947,16 @@
       <c r="O20" s="17" t="s">
         <v>228</v>
       </c>
-      <c r="P20" s="63" t="s">
+      <c r="P20" s="62" t="s">
         <v>219</v>
       </c>
       <c r="Q20" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="R20" s="65" t="s">
+      <c r="R20" s="64" t="s">
         <v>283</v>
       </c>
-      <c r="S20" s="35" t="s">
+      <c r="S20" s="34" t="s">
         <v>284</v>
       </c>
       <c r="T20" s="19" t="s">
@@ -6883,64 +6977,64 @@
       <c r="Y20" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="Z20" s="63" t="s">
+      <c r="Z20" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="AA20" s="59" t="s">
+      <c r="AA20" s="58" t="s">
         <v>202</v>
       </c>
-      <c r="AB20" s="63" t="s">
+      <c r="AB20" s="62" t="s">
         <v>126</v>
       </c>
-      <c r="AC20" s="59" t="s">
+      <c r="AC20" s="58" t="s">
         <v>220</v>
       </c>
-      <c r="AD20" s="58" t="s">
+      <c r="AD20" s="57" t="s">
         <v>233</v>
       </c>
-      <c r="AE20" s="59" t="s">
+      <c r="AE20" s="58" t="s">
         <v>182</v>
       </c>
-      <c r="AF20" s="66" t="s">
+      <c r="AF20" s="65" t="s">
         <v>125</v>
       </c>
       <c r="AG20" s="16" t="s">
         <v>198</v>
       </c>
-      <c r="AH20" s="50" t="s">
+      <c r="AH20" s="49" t="s">
         <v>289</v>
       </c>
-      <c r="AI20" s="36" t="s">
+      <c r="AI20" s="35" t="s">
         <v>290</v>
       </c>
-      <c r="AJ20" s="50" t="s">
+      <c r="AJ20" s="49" t="s">
         <v>291</v>
       </c>
-      <c r="AK20" s="36" t="s">
+      <c r="AK20" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="AL20" s="50" t="s">
+      <c r="AL20" s="49" t="s">
         <v>292</v>
       </c>
-      <c r="AM20" s="36" t="s">
+      <c r="AM20" s="35" t="s">
         <v>293</v>
       </c>
-      <c r="AN20" s="50" t="s">
+      <c r="AN20" s="49" t="s">
         <v>330</v>
       </c>
-      <c r="AO20" s="36" t="s">
+      <c r="AO20" s="35" t="s">
         <v>295</v>
       </c>
-      <c r="AP20" s="50" t="s">
+      <c r="AP20" s="49" t="s">
         <v>331</v>
       </c>
-      <c r="AQ20" s="36" t="s">
+      <c r="AQ20" s="35" t="s">
         <v>332</v>
       </c>
-      <c r="AR20" s="50" t="s">
+      <c r="AR20" s="49" t="s">
         <v>333</v>
       </c>
-      <c r="AS20" s="36" t="s">
+      <c r="AS20" s="35" t="s">
         <v>326</v>
       </c>
       <c r="AT20" s="16" t="s">
@@ -7032,11 +7126,11 @@
       <c r="Q21" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="R21" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="S21" s="34" t="s">
-        <v>241</v>
+      <c r="R21" s="80" t="s">
+        <v>555</v>
+      </c>
+      <c r="S21" s="81" t="s">
+        <v>155</v>
       </c>
       <c r="T21" s="25" t="s">
         <v>14</v>
@@ -7098,16 +7192,16 @@
       <c r="AM21" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN21" s="57" t="s">
+      <c r="AN21" s="56" t="s">
         <v>334</v>
       </c>
-      <c r="AO21" s="36" t="s">
+      <c r="AO21" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="AP21" s="57" t="s">
+      <c r="AP21" s="56" t="s">
         <v>335</v>
       </c>
-      <c r="AQ21" s="36" t="s">
+      <c r="AQ21" s="35" t="s">
         <v>336</v>
       </c>
       <c r="AR21" s="16" t="s">
@@ -7253,10 +7347,10 @@
       <c r="AG22" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AH22" s="52" t="s">
+      <c r="AH22" s="51" t="s">
         <v>286</v>
       </c>
-      <c r="AI22" s="36" t="s">
+      <c r="AI22" s="35" t="s">
         <v>173</v>
       </c>
       <c r="AJ22" s="16" t="s">
@@ -7271,10 +7365,10 @@
       <c r="AM22" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="AN22" s="52" t="s">
+      <c r="AN22" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="AO22" s="36" t="s">
+      <c r="AO22" s="35" t="s">
         <v>226</v>
       </c>
       <c r="AP22" s="16" t="s">
@@ -7564,1258 +7658,1258 @@
   <dimension ref="A1:L66"/>
   <sheetFormatPr defaultColWidth="2.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.77734375" style="37" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.21875" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31" style="37" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.21875" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" style="37" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" style="37" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="2.6640625" style="37"/>
+    <col min="1" max="1" width="29.77734375" style="36" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" style="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.21875" style="36" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" style="36" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31" style="36" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="36" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.109375" style="36" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.21875" style="36" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" style="36" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7" style="36" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="36" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" style="36" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="2.6640625" style="36"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74" t="s">
+      <c r="B1" s="82"/>
+      <c r="C1" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74" t="s">
+      <c r="D1" s="82"/>
+      <c r="E1" s="82" t="s">
         <v>218</v>
       </c>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74" t="s">
+      <c r="F1" s="82"/>
+      <c r="G1" s="82" t="s">
         <v>435</v>
       </c>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74" t="s">
+      <c r="H1" s="82"/>
+      <c r="I1" s="82" t="s">
         <v>516</v>
       </c>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="37" t="s">
         <v>337</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="37" t="s">
         <v>405</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="37" t="s">
         <v>337</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="37" t="s">
         <v>405</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="37" t="s">
         <v>337</v>
       </c>
-      <c r="F2" s="38" t="s">
+      <c r="F2" s="37" t="s">
         <v>405</v>
       </c>
-      <c r="G2" s="38" t="s">
+      <c r="G2" s="37" t="s">
         <v>455</v>
       </c>
-      <c r="H2" s="38" t="s">
+      <c r="H2" s="37" t="s">
         <v>454</v>
       </c>
-      <c r="I2" s="38" t="s">
+      <c r="I2" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="38" t="s">
+      <c r="J2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="38" t="s">
+      <c r="K2" s="37" t="s">
         <v>218</v>
       </c>
-      <c r="L2" s="38" t="s">
+      <c r="L2" s="37" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="36" t="s">
         <v>338</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="36" t="s">
         <v>339</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="36" t="s">
         <v>340</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="D3" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="36" t="s">
         <v>341</v>
       </c>
-      <c r="F3" s="37" t="s">
+      <c r="F3" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G3" s="44" t="s">
+      <c r="G3" s="43" t="s">
         <v>436</v>
       </c>
-      <c r="H3" s="37" t="s">
+      <c r="H3" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="72" t="s">
+      <c r="I3" s="71" t="s">
         <v>385</v>
       </c>
-      <c r="J3" s="71" t="s">
+      <c r="J3" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="71" t="s">
+      <c r="K3" s="70" t="s">
         <v>366</v>
       </c>
-      <c r="L3" s="71" t="s">
+      <c r="L3" s="70" t="s">
         <v>517</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>343</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="36" t="s">
         <v>339</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="36" t="s">
         <v>344</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="36" t="s">
         <v>345</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="43" t="s">
         <v>456</v>
       </c>
-      <c r="H4" s="44" t="s">
+      <c r="H4" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="71" t="s">
+      <c r="I4" s="70" t="s">
         <v>347</v>
       </c>
-      <c r="J4" s="71" t="s">
+      <c r="J4" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="K4" s="71" t="s">
+      <c r="K4" s="70" t="s">
         <v>366</v>
       </c>
-      <c r="L4" s="71" t="s">
+      <c r="L4" s="70" t="s">
         <v>518</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="36" t="s">
         <v>346</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="36" t="s">
         <v>348</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="36" t="s">
         <v>349</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G5" s="44" t="s">
+      <c r="G5" s="43" t="s">
         <v>457</v>
       </c>
-      <c r="H5" s="44" t="s">
+      <c r="H5" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="71" t="s">
+      <c r="I5" s="70" t="s">
         <v>519</v>
       </c>
-      <c r="J5" s="71" t="s">
+      <c r="J5" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="71" t="s">
+      <c r="K5" s="70" t="s">
         <v>366</v>
       </c>
-      <c r="L5" s="71" t="s">
+      <c r="L5" s="70" t="s">
         <v>520</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="36" t="s">
         <v>350</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="36" t="s">
         <v>351</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="D6" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="36" t="s">
         <v>352</v>
       </c>
-      <c r="F6" s="37" t="s">
+      <c r="F6" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="37" t="s">
+      <c r="I6" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="J6" s="71" t="s">
+      <c r="J6" s="70" t="s">
         <v>284</v>
       </c>
-      <c r="K6" s="71" t="s">
+      <c r="K6" s="70" t="s">
         <v>366</v>
       </c>
-      <c r="L6" s="71" t="s">
+      <c r="L6" s="70" t="s">
         <v>521</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="36" t="s">
         <v>353</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="E7" s="36" t="s">
         <v>355</v>
       </c>
-      <c r="F7" s="37" t="s">
+      <c r="F7" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="H7" s="45" t="s">
+      <c r="H7" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="I7" s="37" t="s">
+      <c r="I7" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="J7" s="71" t="s">
+      <c r="J7" s="70" t="s">
         <v>284</v>
       </c>
-      <c r="K7" s="71" t="s">
+      <c r="K7" s="70" t="s">
         <v>366</v>
       </c>
-      <c r="L7" s="71" t="s">
+      <c r="L7" s="70" t="s">
         <v>522</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="36" t="s">
         <v>356</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="D8" s="37" t="s">
+      <c r="D8" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E8" s="37" t="s">
+      <c r="E8" s="36" t="s">
         <v>357</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="43" t="s">
         <v>459</v>
       </c>
-      <c r="H8" s="44" t="s">
+      <c r="H8" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="I8" s="37" t="s">
+      <c r="I8" s="36" t="s">
         <v>519</v>
       </c>
-      <c r="J8" s="71" t="s">
+      <c r="J8" s="70" t="s">
         <v>284</v>
       </c>
-      <c r="K8" s="71" t="s">
+      <c r="K8" s="70" t="s">
         <v>366</v>
       </c>
-      <c r="L8" s="71" t="s">
+      <c r="L8" s="70" t="s">
         <v>523</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="36" t="s">
         <v>358</v>
       </c>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="36" t="s">
         <v>401</v>
       </c>
-      <c r="D9" s="37" t="s">
+      <c r="D9" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="36" t="s">
         <v>360</v>
       </c>
-      <c r="F9" s="37" t="s">
+      <c r="F9" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G9" s="44" t="s">
+      <c r="G9" s="43" t="s">
         <v>437</v>
       </c>
-      <c r="H9" s="37" t="s">
+      <c r="H9" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="37" t="s">
+      <c r="I9" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="J9" s="71" t="s">
+      <c r="J9" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="71" t="s">
+      <c r="K9" s="70" t="s">
         <v>342</v>
       </c>
-      <c r="L9" s="71" t="s">
+      <c r="L9" s="70" t="s">
         <v>524</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="36" t="s">
         <v>361</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="36" t="s">
         <v>359</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="36" t="s">
         <v>363</v>
       </c>
-      <c r="F10" s="37" t="s">
+      <c r="F10" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G10" s="44" t="s">
+      <c r="G10" s="43" t="s">
         <v>475</v>
       </c>
-      <c r="H10" s="37" t="s">
+      <c r="H10" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="I10" s="37" t="s">
+      <c r="I10" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="J10" s="71" t="s">
+      <c r="J10" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="K10" s="71" t="s">
+      <c r="K10" s="70" t="s">
         <v>342</v>
       </c>
-      <c r="L10" s="71" t="s">
+      <c r="L10" s="70" t="s">
         <v>525</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="36" t="s">
         <v>364</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="36" t="s">
         <v>362</v>
       </c>
-      <c r="D11" s="37" t="s">
+      <c r="D11" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="37" t="s">
+      <c r="E11" s="36" t="s">
         <v>400</v>
       </c>
-      <c r="F11" s="37" t="s">
+      <c r="F11" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="37" t="s">
+      <c r="H11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="37" t="s">
+      <c r="I11" s="36" t="s">
         <v>519</v>
       </c>
-      <c r="J11" s="71" t="s">
+      <c r="J11" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="K11" s="71" t="s">
+      <c r="K11" s="70" t="s">
         <v>342</v>
       </c>
-      <c r="L11" s="71" t="s">
+      <c r="L11" s="70" t="s">
         <v>526</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="36" t="s">
         <v>367</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="36" t="s">
         <v>365</v>
       </c>
-      <c r="D12" s="37" t="s">
+      <c r="D12" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="37" t="s">
+      <c r="E12" s="36" t="s">
         <v>377</v>
       </c>
-      <c r="F12" s="44" t="s">
+      <c r="F12" s="43" t="s">
         <v>342</v>
       </c>
-      <c r="G12" s="45" t="s">
+      <c r="G12" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="H12" s="37" t="s">
+      <c r="H12" s="36" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="36" t="s">
         <v>369</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C13" s="37" t="s">
+      <c r="C13" s="36" t="s">
         <v>368</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="37" t="s">
+      <c r="E13" s="36" t="s">
         <v>383</v>
       </c>
-      <c r="F13" s="45" t="s">
+      <c r="F13" s="44" t="s">
         <v>342</v>
       </c>
-      <c r="G13" s="44" t="s">
+      <c r="G13" s="43" t="s">
         <v>458</v>
       </c>
-      <c r="H13" s="44" t="s">
+      <c r="H13" s="43" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="36" t="s">
         <v>371</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="36" t="s">
         <v>357</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="D14" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="37" t="s">
+      <c r="E14" s="36" t="s">
         <v>348</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="F14" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G14" s="45" t="s">
+      <c r="G14" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="H14" s="37" t="s">
+      <c r="H14" s="36" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="36" t="s">
         <v>373</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="36" t="s">
         <v>369</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D15" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="37" t="s">
+      <c r="E15" s="36" t="s">
         <v>369</v>
       </c>
-      <c r="F15" s="37" t="s">
+      <c r="F15" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G15" s="44" t="s">
+      <c r="G15" s="43" t="s">
         <v>132</v>
       </c>
-      <c r="H15" s="37" t="s">
+      <c r="H15" s="36" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="36" t="s">
         <v>375</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="36" t="s">
         <v>370</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="37" t="s">
+      <c r="E16" s="36" t="s">
         <v>370</v>
       </c>
-      <c r="F16" s="37" t="s">
+      <c r="F16" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G16" s="44" t="s">
+      <c r="G16" s="43" t="s">
         <v>460</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="43" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="36" t="s">
         <v>377</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C17" s="37" t="s">
+      <c r="C17" s="36" t="s">
         <v>360</v>
       </c>
-      <c r="D17" s="37" t="s">
+      <c r="D17" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="37" t="s">
+      <c r="E17" s="36" t="s">
         <v>372</v>
       </c>
-      <c r="F17" s="37" t="s">
+      <c r="F17" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G17" s="44" t="s">
+      <c r="G17" s="43" t="s">
         <v>438</v>
       </c>
-      <c r="H17" s="37" t="s">
+      <c r="H17" s="36" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="36" t="s">
         <v>380</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C18" s="37" t="s">
+      <c r="C18" s="36" t="s">
         <v>378</v>
       </c>
-      <c r="D18" s="37" t="s">
+      <c r="D18" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="37" t="s">
+      <c r="E18" s="36" t="s">
         <v>374</v>
       </c>
-      <c r="F18" s="37" t="s">
+      <c r="F18" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G18" s="44" t="s">
+      <c r="G18" s="43" t="s">
         <v>461</v>
       </c>
-      <c r="H18" s="44" t="s">
+      <c r="H18" s="43" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="36" t="s">
         <v>357</v>
       </c>
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C19" s="37" t="s">
+      <c r="C19" s="36" t="s">
         <v>363</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="36" t="s">
         <v>376</v>
       </c>
-      <c r="F19" s="37" t="s">
+      <c r="F19" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G19" s="44" t="s">
+      <c r="G19" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="H19" s="44" t="s">
+      <c r="H19" s="43" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="37" t="s">
+      <c r="A20" s="36" t="s">
         <v>382</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C20" s="37" t="s">
+      <c r="C20" s="36" t="s">
         <v>399</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="D20" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="37" t="s">
+      <c r="E20" s="36" t="s">
         <v>379</v>
       </c>
-      <c r="F20" s="37" t="s">
+      <c r="F20" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G20" s="44" t="s">
+      <c r="G20" s="43" t="s">
         <v>439</v>
       </c>
-      <c r="H20" s="37" t="s">
+      <c r="H20" s="36" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="36" t="s">
         <v>383</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C21" s="37" t="s">
+      <c r="C21" s="36" t="s">
         <v>400</v>
       </c>
-      <c r="D21" s="37" t="s">
+      <c r="D21" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="37" t="s">
+      <c r="E21" s="36" t="s">
         <v>381</v>
       </c>
-      <c r="F21" s="37" t="s">
+      <c r="F21" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G21" s="44" t="s">
+      <c r="G21" s="43" t="s">
         <v>462</v>
       </c>
-      <c r="H21" s="44" t="s">
+      <c r="H21" s="43" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="36" t="s">
         <v>360</v>
       </c>
-      <c r="B22" s="37" t="s">
+      <c r="B22" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="36" t="s">
         <v>380</v>
       </c>
-      <c r="D22" s="44" t="s">
+      <c r="D22" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="E22" s="37" t="s">
+      <c r="E22" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="F22" s="37" t="s">
+      <c r="F22" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G22" s="44" t="s">
+      <c r="G22" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="H22" s="44" t="s">
+      <c r="H22" s="43" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="37" t="s">
+      <c r="A23" s="36" t="s">
         <v>378</v>
       </c>
-      <c r="B23" s="37" t="s">
+      <c r="B23" s="36" t="s">
         <v>347</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="C23" s="36" t="s">
         <v>377</v>
       </c>
-      <c r="D23" s="44" t="s">
+      <c r="D23" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="37" t="s">
+      <c r="E23" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="F23" s="37" t="s">
+      <c r="F23" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G23" s="37" t="s">
+      <c r="G23" s="36" t="s">
         <v>135</v>
       </c>
-      <c r="H23" s="37" t="s">
+      <c r="H23" s="36" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="38" t="s">
         <v>384</v>
       </c>
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="C24" s="37" t="s">
+      <c r="C24" s="36" t="s">
         <v>483</v>
       </c>
-      <c r="D24" s="37" t="s">
+      <c r="D24" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="37" t="s">
+      <c r="E24" s="36" t="s">
         <v>378</v>
       </c>
-      <c r="F24" s="37" t="s">
+      <c r="F24" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G24" s="44" t="s">
+      <c r="G24" s="43" t="s">
         <v>440</v>
       </c>
-      <c r="H24" s="37" t="s">
+      <c r="H24" s="36" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="39" t="s">
+      <c r="A25" s="38" t="s">
         <v>386</v>
       </c>
-      <c r="B25" s="37" t="s">
+      <c r="B25" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="E25" s="37" t="s">
+      <c r="E25" s="36" t="s">
         <v>399</v>
       </c>
-      <c r="F25" s="37" t="s">
+      <c r="F25" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G25" s="44" t="s">
+      <c r="G25" s="43" t="s">
         <v>463</v>
       </c>
-      <c r="H25" s="44" t="s">
+      <c r="H25" s="43" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="39" t="s">
+      <c r="A26" s="38" t="s">
         <v>387</v>
       </c>
-      <c r="B26" s="37" t="s">
+      <c r="B26" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="E26" s="37" t="s">
+      <c r="E26" s="36" t="s">
         <v>401</v>
       </c>
-      <c r="F26" s="37" t="s">
+      <c r="F26" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="G26" s="44" t="s">
+      <c r="G26" s="43" t="s">
         <v>441</v>
       </c>
-      <c r="H26" s="37" t="s">
+      <c r="H26" s="36" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="39" t="s">
+      <c r="A27" s="38" t="s">
         <v>388</v>
       </c>
-      <c r="B27" s="37" t="s">
+      <c r="B27" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="E27" s="37" t="s">
+      <c r="E27" s="36" t="s">
         <v>380</v>
       </c>
-      <c r="F27" s="44" t="s">
+      <c r="F27" s="43" t="s">
         <v>366</v>
       </c>
-      <c r="G27" s="44" t="s">
+      <c r="G27" s="43" t="s">
         <v>464</v>
       </c>
-      <c r="H27" s="44" t="s">
+      <c r="H27" s="43" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="38" t="s">
         <v>389</v>
       </c>
-      <c r="B28" s="37" t="s">
+      <c r="B28" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="E28" s="37" t="s">
+      <c r="E28" s="36" t="s">
         <v>387</v>
       </c>
-      <c r="F28" s="45" t="s">
+      <c r="F28" s="44" t="s">
         <v>366</v>
       </c>
-      <c r="G28" s="44" t="s">
+      <c r="G28" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="H28" s="44" t="s">
+      <c r="H28" s="43" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="39" t="s">
+      <c r="A29" s="38" t="s">
         <v>390</v>
       </c>
-      <c r="B29" s="37" t="s">
+      <c r="B29" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="E29" s="37" t="s">
+      <c r="E29" s="36" t="s">
         <v>350</v>
       </c>
-      <c r="F29" s="45" t="s">
+      <c r="F29" s="44" t="s">
         <v>366</v>
       </c>
-      <c r="G29" s="37" t="s">
+      <c r="G29" s="36" t="s">
         <v>137</v>
       </c>
-      <c r="H29" s="37" t="s">
+      <c r="H29" s="36" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="39" t="s">
+      <c r="A30" s="38" t="s">
         <v>391</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="B30" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G30" s="44" t="s">
+      <c r="G30" s="43" t="s">
         <v>442</v>
       </c>
-      <c r="H30" s="37" t="s">
+      <c r="H30" s="36" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="39" t="s">
+      <c r="A31" s="38" t="s">
         <v>392</v>
       </c>
-      <c r="B31" s="37" t="s">
+      <c r="B31" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G31" s="44" t="s">
+      <c r="G31" s="43" t="s">
         <v>473</v>
       </c>
-      <c r="H31" s="44" t="s">
+      <c r="H31" s="43" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="38" t="s">
         <v>393</v>
       </c>
-      <c r="B32" s="37" t="s">
+      <c r="B32" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G32" s="44" t="s">
+      <c r="G32" s="43" t="s">
         <v>453</v>
       </c>
-      <c r="H32" s="37" t="s">
+      <c r="H32" s="36" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="39" t="s">
+      <c r="A33" s="38" t="s">
         <v>394</v>
       </c>
-      <c r="B33" s="37" t="s">
+      <c r="B33" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G33" s="44" t="s">
+      <c r="G33" s="43" t="s">
         <v>445</v>
       </c>
-      <c r="H33" s="44" t="s">
+      <c r="H33" s="43" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="39" t="s">
+      <c r="A34" s="38" t="s">
         <v>395</v>
       </c>
-      <c r="B34" s="37" t="s">
+      <c r="B34" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G34" s="44" t="s">
+      <c r="G34" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="H34" s="44" t="s">
+      <c r="H34" s="43" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="39" t="s">
+      <c r="A35" s="38" t="s">
         <v>396</v>
       </c>
-      <c r="B35" s="37" t="s">
+      <c r="B35" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G35" s="37" t="s">
+      <c r="G35" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="H35" s="37" t="s">
+      <c r="H35" s="36" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="39" t="s">
+      <c r="A36" s="38" t="s">
         <v>370</v>
       </c>
-      <c r="B36" s="37" t="s">
+      <c r="B36" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G36" s="44" t="s">
+      <c r="G36" s="43" t="s">
         <v>443</v>
       </c>
-      <c r="H36" s="37" t="s">
+      <c r="H36" s="36" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="39" t="s">
+      <c r="A37" s="38" t="s">
         <v>348</v>
       </c>
-      <c r="B37" s="37" t="s">
+      <c r="B37" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G37" s="44" t="s">
+      <c r="G37" s="43" t="s">
         <v>465</v>
       </c>
-      <c r="H37" s="44" t="s">
+      <c r="H37" s="43" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="39" t="s">
+      <c r="A38" s="38" t="s">
         <v>397</v>
       </c>
-      <c r="B38" s="37" t="s">
+      <c r="B38" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G38" s="44" t="s">
+      <c r="G38" s="43" t="s">
         <v>476</v>
       </c>
-      <c r="H38" s="44" t="s">
+      <c r="H38" s="43" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="39" t="s">
+      <c r="A39" s="38" t="s">
         <v>398</v>
       </c>
-      <c r="B39" s="37" t="s">
+      <c r="B39" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G39" s="44" t="s">
+      <c r="G39" s="43" t="s">
         <v>444</v>
       </c>
-      <c r="H39" s="37" t="s">
+      <c r="H39" s="36" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="38" t="s">
         <v>399</v>
       </c>
-      <c r="B40" s="37" t="s">
+      <c r="B40" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G40" s="44" t="s">
+      <c r="G40" s="43" t="s">
         <v>466</v>
       </c>
-      <c r="H40" s="44" t="s">
+      <c r="H40" s="43" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="39" t="s">
+      <c r="A41" s="38" t="s">
         <v>400</v>
       </c>
-      <c r="B41" s="37" t="s">
+      <c r="B41" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G41" s="44" t="s">
+      <c r="G41" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="H41" s="44" t="s">
+      <c r="H41" s="43" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="39" t="s">
+      <c r="A42" s="38" t="s">
         <v>401</v>
       </c>
-      <c r="B42" s="37" t="s">
+      <c r="B42" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G42" s="37" t="s">
+      <c r="G42" s="36" t="s">
         <v>141</v>
       </c>
-      <c r="H42" s="37" t="s">
+      <c r="H42" s="36" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="37" t="s">
+      <c r="A43" s="36" t="s">
         <v>363</v>
       </c>
-      <c r="B43" s="37" t="s">
+      <c r="B43" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G43" s="44" t="s">
+      <c r="G43" s="43" t="s">
         <v>446</v>
       </c>
-      <c r="H43" s="37" t="s">
+      <c r="H43" s="36" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="37" t="s">
+      <c r="A44" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="B44" s="37" t="s">
+      <c r="B44" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G44" s="44" t="s">
+      <c r="G44" s="43" t="s">
         <v>467</v>
       </c>
-      <c r="H44" s="44" t="s">
+      <c r="H44" s="43" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="37" t="s">
+      <c r="A45" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="B45" s="37" t="s">
+      <c r="B45" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G45" s="44" t="s">
+      <c r="G45" s="43" t="s">
         <v>447</v>
       </c>
-      <c r="H45" s="37" t="s">
+      <c r="H45" s="36" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="37" t="s">
+      <c r="A46" s="36" t="s">
         <v>515</v>
       </c>
-      <c r="B46" s="37" t="s">
+      <c r="B46" s="36" t="s">
         <v>385</v>
       </c>
-      <c r="G46" s="44" t="s">
+      <c r="G46" s="43" t="s">
         <v>468</v>
       </c>
-      <c r="H46" s="44" t="s">
+      <c r="H46" s="43" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G47" s="44" t="s">
+      <c r="G47" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="H47" s="44" t="s">
+      <c r="H47" s="43" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G48" s="37" t="s">
+      <c r="G48" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="H48" s="37" t="s">
+      <c r="H48" s="36" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="49" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G49" s="44" t="s">
+      <c r="G49" s="43" t="s">
         <v>448</v>
       </c>
-      <c r="H49" s="37" t="s">
+      <c r="H49" s="36" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="50" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G50" s="44" t="s">
+      <c r="G50" s="43" t="s">
         <v>469</v>
       </c>
-      <c r="H50" s="44" t="s">
+      <c r="H50" s="43" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="51" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G51" s="44" t="s">
+      <c r="G51" s="43" t="s">
         <v>449</v>
       </c>
-      <c r="H51" s="37" t="s">
+      <c r="H51" s="36" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="52" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G52" s="44" t="s">
+      <c r="G52" s="43" t="s">
         <v>470</v>
       </c>
-      <c r="H52" s="44" t="s">
+      <c r="H52" s="43" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="53" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G53" s="44" t="s">
+      <c r="G53" s="43" t="s">
         <v>144</v>
       </c>
-      <c r="H53" s="44" t="s">
+      <c r="H53" s="43" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="54" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G54" s="37" t="s">
+      <c r="G54" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="H54" s="37" t="s">
+      <c r="H54" s="36" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="55" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G55" s="44" t="s">
+      <c r="G55" s="43" t="s">
         <v>450</v>
       </c>
-      <c r="H55" s="37" t="s">
+      <c r="H55" s="36" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="56" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G56" s="44" t="s">
+      <c r="G56" s="43" t="s">
         <v>471</v>
       </c>
-      <c r="H56" s="44" t="s">
+      <c r="H56" s="43" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="57" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G57" s="44" t="s">
+      <c r="G57" s="43" t="s">
         <v>451</v>
       </c>
-      <c r="H57" s="37" t="s">
+      <c r="H57" s="36" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="58" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G58" s="37" t="s">
+      <c r="G58" s="36" t="s">
         <v>242</v>
       </c>
-      <c r="H58" s="37" t="s">
+      <c r="H58" s="36" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="59" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G59" s="37" t="s">
+      <c r="G59" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="H59" s="37" t="s">
+      <c r="H59" s="36" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="60" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G60" s="44" t="s">
+      <c r="G60" s="43" t="s">
         <v>452</v>
       </c>
-      <c r="H60" s="37" t="s">
+      <c r="H60" s="36" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="61" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G61" s="44" t="s">
+      <c r="G61" s="43" t="s">
         <v>472</v>
       </c>
-      <c r="H61" s="44" t="s">
+      <c r="H61" s="43" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="62" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G62" s="45" t="s">
+      <c r="G62" s="44" t="s">
         <v>478</v>
       </c>
-      <c r="H62" s="45" t="s">
+      <c r="H62" s="44" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="63" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G63" s="37" t="s">
+      <c r="G63" s="36" t="s">
         <v>479</v>
       </c>
-      <c r="H63" s="45" t="s">
+      <c r="H63" s="44" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="64" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G64" s="45" t="s">
+      <c r="G64" s="44" t="s">
         <v>480</v>
       </c>
-      <c r="H64" s="45" t="s">
+      <c r="H64" s="44" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="65" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G65" s="37" t="s">
+      <c r="G65" s="36" t="s">
         <v>481</v>
       </c>
-      <c r="H65" s="45" t="s">
+      <c r="H65" s="44" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="66" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G66" s="45" t="s">
+      <c r="G66" s="44" t="s">
         <v>482</v>
       </c>
-      <c r="H66" s="45" t="s">
+      <c r="H66" s="44" t="s">
         <v>137</v>
       </c>
     </row>
@@ -8839,588 +8933,588 @@
   <dimension ref="A1:B88"/>
   <sheetFormatPr defaultColWidth="5.44140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.44140625" style="42"/>
-    <col min="2" max="2" width="204.88671875" style="40" customWidth="1"/>
-    <col min="3" max="16384" width="5.44140625" style="40"/>
+    <col min="1" max="1" width="5.44140625" style="41"/>
+    <col min="2" max="2" width="204.88671875" style="39" customWidth="1"/>
+    <col min="3" max="16384" width="5.44140625" style="39"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="42" t="s">
+    <row r="1" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="41" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42">
+      <c r="A2" s="41">
         <v>1</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="39" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42">
+      <c r="A3" s="41">
         <v>2</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="39" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="42">
+      <c r="A4" s="41">
         <v>3</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="39" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="42">
+      <c r="A5" s="41">
         <v>4</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="39" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="42">
+      <c r="A6" s="41">
         <v>5</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="39" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="42">
+      <c r="A7" s="41">
         <v>6</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="39" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="42">
+      <c r="A8" s="41">
         <v>7</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="39" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="42">
+      <c r="A9" s="41">
         <v>8</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="39" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="42" t="s">
+    <row r="11" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="41" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="42">
+      <c r="A12" s="41">
         <v>1</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="39" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="42">
+      <c r="A13" s="41">
         <v>2</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="39" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="42">
+      <c r="A14" s="41">
         <v>3</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="39" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="42">
+      <c r="A15" s="41">
         <v>4</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="39" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="42">
+      <c r="A16" s="41">
         <v>5</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="39" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="42">
+      <c r="A17" s="41">
         <v>6</v>
       </c>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="39" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="42">
+      <c r="A18" s="41">
         <v>7</v>
       </c>
-      <c r="B18" s="40" t="s">
+      <c r="B18" s="39" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="42">
+      <c r="A19" s="41">
         <v>8</v>
       </c>
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="39" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="42">
+      <c r="A20" s="41">
         <v>9</v>
       </c>
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="39" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="42">
+      <c r="A21" s="41">
         <v>10</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="39" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="42">
+      <c r="A22" s="41">
         <v>11</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="39" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="42">
+      <c r="A23" s="41">
         <v>12</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="39" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="42">
+      <c r="A24" s="41">
         <v>13</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="39" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="42">
+      <c r="A25" s="41">
         <v>14</v>
       </c>
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="39" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="42">
+      <c r="A26" s="41">
         <v>15</v>
       </c>
-      <c r="B26" s="40" t="s">
+      <c r="B26" s="39" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="28" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="42" t="s">
+    <row r="28" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="41" t="s">
         <v>425</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="42">
+      <c r="A29" s="41">
         <v>1</v>
       </c>
-      <c r="B29" s="40" t="s">
+      <c r="B29" s="39" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="42">
+      <c r="A30" s="41">
         <v>2</v>
       </c>
-      <c r="B30" s="40" t="s">
+      <c r="B30" s="39" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="42">
+      <c r="A31" s="41">
         <v>3</v>
       </c>
-      <c r="B31" s="40" t="s">
+      <c r="B31" s="39" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="42">
+      <c r="A32" s="41">
         <v>4</v>
       </c>
-      <c r="B32" s="40" t="s">
+      <c r="B32" s="39" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="42">
+      <c r="A33" s="41">
         <v>5</v>
       </c>
-      <c r="B33" s="40" t="s">
+      <c r="B33" s="39" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="42">
+      <c r="A34" s="41">
         <v>6</v>
       </c>
-      <c r="B34" s="40" t="s">
+      <c r="B34" s="39" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="42">
+      <c r="A35" s="41">
         <v>7</v>
       </c>
-      <c r="B35" s="40" t="s">
+      <c r="B35" s="39" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="42">
+      <c r="A36" s="41">
         <v>8</v>
       </c>
-      <c r="B36" s="40" t="s">
+      <c r="B36" s="39" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="42">
+      <c r="A37" s="41">
         <v>9</v>
       </c>
-      <c r="B37" s="41" t="s">
+      <c r="B37" s="40" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="42">
+      <c r="A38" s="41">
         <v>10</v>
       </c>
-      <c r="B38" s="40" t="s">
+      <c r="B38" s="39" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="42">
+      <c r="A39" s="41">
         <v>11</v>
       </c>
-      <c r="B39" s="40" t="s">
+      <c r="B39" s="39" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="41" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="42" t="s">
+    <row r="41" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="41" t="s">
         <v>426</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="42">
+      <c r="A42" s="41">
         <v>1</v>
       </c>
-      <c r="B42" s="40" t="s">
+      <c r="B42" s="39" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="42">
+      <c r="A43" s="41">
         <v>2</v>
       </c>
-      <c r="B43" s="40" t="s">
+      <c r="B43" s="39" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="42">
+      <c r="A44" s="41">
         <v>3</v>
       </c>
-      <c r="B44" s="40" t="s">
+      <c r="B44" s="39" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="42">
+      <c r="A45" s="41">
         <v>4</v>
       </c>
-      <c r="B45" s="40" t="s">
+      <c r="B45" s="39" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="42">
+      <c r="A46" s="41">
         <v>5</v>
       </c>
-      <c r="B46" s="40" t="s">
+      <c r="B46" s="39" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="42">
+      <c r="A47" s="41">
         <v>6</v>
       </c>
-      <c r="B47" s="40" t="s">
+      <c r="B47" s="39" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="42">
+      <c r="A48" s="41">
         <v>7</v>
       </c>
-      <c r="B48" s="40" t="s">
+      <c r="B48" s="39" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="42">
+      <c r="A49" s="41">
         <v>8</v>
       </c>
-      <c r="B49" s="40" t="s">
+      <c r="B49" s="39" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="51" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="42" t="s">
+    <row r="51" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="41" t="s">
         <v>427</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="42">
+      <c r="A52" s="41">
         <v>1</v>
       </c>
-      <c r="B52" s="40" t="s">
+      <c r="B52" s="39" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="42">
+      <c r="A53" s="41">
         <v>2</v>
       </c>
-      <c r="B53" s="40" t="s">
+      <c r="B53" s="39" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="42">
+      <c r="A54" s="41">
         <v>3</v>
       </c>
-      <c r="B54" s="40" t="s">
+      <c r="B54" s="39" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="42">
+      <c r="A55" s="41">
         <v>4</v>
       </c>
-      <c r="B55" s="40" t="s">
+      <c r="B55" s="39" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="57" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="42" t="s">
+    <row r="57" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="41" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="42">
+      <c r="A58" s="41">
         <v>1</v>
       </c>
-      <c r="B58" s="40" t="s">
+      <c r="B58" s="39" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="60" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="42" t="s">
+    <row r="60" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="41" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="42">
+      <c r="A61" s="41">
         <v>1</v>
       </c>
-      <c r="B61" s="40" t="s">
+      <c r="B61" s="39" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="42">
+      <c r="A62" s="41">
         <v>2</v>
       </c>
-      <c r="B62" s="40" t="s">
+      <c r="B62" s="39" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="42">
+      <c r="A63" s="41">
         <v>3</v>
       </c>
-      <c r="B63" s="40" t="s">
+      <c r="B63" s="39" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A64" s="42">
+      <c r="A64" s="41">
         <v>4</v>
       </c>
-      <c r="B64" s="40" t="s">
+      <c r="B64" s="39" t="s">
         <v>406</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="42">
+      <c r="A65" s="41">
         <v>5</v>
       </c>
-      <c r="B65" s="40" t="s">
+      <c r="B65" s="39" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="67" spans="1:2" s="42" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="42" t="s">
+    <row r="67" spans="1:2" s="41" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="41" t="s">
         <v>430</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="42">
+      <c r="A68" s="41">
         <v>1</v>
       </c>
-      <c r="B68" s="40" t="s">
+      <c r="B68" s="39" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="42">
+      <c r="A69" s="41">
         <v>2</v>
       </c>
-      <c r="B69" s="40" t="s">
+      <c r="B69" s="39" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="42">
+      <c r="A70" s="41">
         <v>3</v>
       </c>
-      <c r="B70" s="43" t="s">
+      <c r="B70" s="42" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="42" t="s">
+      <c r="B72" s="41" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="42">
+      <c r="A73" s="41">
         <v>1</v>
       </c>
-      <c r="B73" s="43" t="s">
+      <c r="B73" s="42" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="42" t="s">
+      <c r="B75" s="41" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="42">
+      <c r="A76" s="41">
         <v>1</v>
       </c>
-      <c r="B76" s="46" t="s">
+      <c r="B76" s="45" t="s">
         <v>477</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="42" t="s">
+      <c r="B78" s="41" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="42">
+      <c r="A79" s="41">
         <v>1</v>
       </c>
-      <c r="B79" s="49" t="s">
+      <c r="B79" s="48" t="s">
         <v>505</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="42">
+      <c r="A80" s="41">
         <v>2</v>
       </c>
-      <c r="B80" s="49" t="s">
+      <c r="B80" s="48" t="s">
         <v>506</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A81" s="42">
+      <c r="A81" s="41">
         <v>3</v>
       </c>
-      <c r="B81" s="67" t="s">
+      <c r="B81" s="66" t="s">
         <v>507</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="42">
+      <c r="A82" s="41">
         <v>4</v>
       </c>
-      <c r="B82" s="67" t="s">
+      <c r="B82" s="66" t="s">
         <v>508</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="42">
+      <c r="A83" s="41">
         <v>5</v>
       </c>
-      <c r="B83" s="67" t="s">
+      <c r="B83" s="66" t="s">
         <v>509</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="42" t="s">
+      <c r="B85" s="41" t="s">
         <v>511</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="42">
+      <c r="A86" s="41">
         <v>1</v>
       </c>
-      <c r="B86" s="70" t="s">
+      <c r="B86" s="69" t="s">
         <v>514</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="42">
+      <c r="A87" s="41">
         <v>2</v>
       </c>
-      <c r="B87" s="67" t="s">
+      <c r="B87" s="66" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="42">
+      <c r="A88" s="41">
         <v>3</v>
       </c>
-      <c r="B88" s="67" t="s">
+      <c r="B88" s="66" t="s">
         <v>513</v>
       </c>
     </row>
@@ -9442,7 +9536,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="72" t="s">
         <v>3</v>
       </c>
       <c r="B1" t="s">
@@ -9678,43 +9772,43 @@
       <c r="A1" t="s">
         <v>552</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="75" t="s">
+      <c r="C1" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="75" t="s">
+      <c r="D1" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="75" t="s">
+      <c r="E1" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="75" t="s">
+      <c r="F1" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="75" t="s">
+      <c r="G1" s="73" t="s">
         <v>547</v>
       </c>
-      <c r="H1" s="75" t="s">
+      <c r="H1" s="73" t="s">
         <v>217</v>
       </c>
-      <c r="I1" s="76" t="s">
+      <c r="I1" s="74" t="s">
         <v>548</v>
       </c>
-      <c r="J1" s="76" t="s">
+      <c r="J1" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="76" t="s">
+      <c r="K1" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="76" t="s">
+      <c r="L1" s="74" t="s">
         <v>549</v>
       </c>
-      <c r="M1" s="76" t="s">
+      <c r="M1" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="76" t="s">
+      <c r="N1" s="74" t="s">
         <v>550</v>
       </c>
     </row>
@@ -9722,256 +9816,256 @@
       <c r="A2" t="s">
         <v>553</v>
       </c>
-      <c r="B2" s="75" t="s">
+      <c r="B2" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="75" t="s">
+      <c r="C2" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="75" t="s">
+      <c r="D2" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="75" t="s">
+      <c r="E2" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="75" t="s">
+      <c r="F2" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="76" t="s">
+      <c r="J2" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="77" t="s">
+      <c r="K2" s="75" t="s">
         <v>551</v>
       </c>
-      <c r="L2" s="76" t="s">
+      <c r="L2" s="74" t="s">
         <v>549</v>
       </c>
-      <c r="M2" s="76" t="s">
+      <c r="M2" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="76" t="s">
+      <c r="N2" s="74" t="s">
         <v>550</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B5" s="79" t="s">
+      <c r="B5" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="79" t="s">
+      <c r="C5" s="77" t="s">
         <v>547</v>
       </c>
-      <c r="D5" s="79" t="s">
+      <c r="D5" s="77" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="78" t="s">
+      <c r="B6" s="76" t="s">
         <v>527</v>
       </c>
-      <c r="C6" s="78"/>
-      <c r="D6" s="78"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="78" t="s">
+      <c r="B7" s="76" t="s">
         <v>528</v>
       </c>
-      <c r="C7" s="78" t="s">
+      <c r="C7" s="76" t="s">
         <v>366</v>
       </c>
-      <c r="D7" s="78" t="s">
+      <c r="D7" s="76" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="78" t="s">
+      <c r="B8" s="76" t="s">
         <v>529</v>
       </c>
-      <c r="C8" s="78" t="s">
+      <c r="C8" s="76" t="s">
         <v>366</v>
       </c>
-      <c r="D8" s="78" t="s">
+      <c r="D8" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B9" s="78" t="s">
+      <c r="B9" s="76" t="s">
         <v>530</v>
       </c>
-      <c r="C9" s="78" t="s">
+      <c r="C9" s="76" t="s">
         <v>342</v>
       </c>
-      <c r="D9" s="78" t="s">
+      <c r="D9" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="78" t="s">
+      <c r="B10" s="76" t="s">
         <v>531</v>
       </c>
-      <c r="C10" s="78" t="s">
+      <c r="C10" s="76" t="s">
         <v>366</v>
       </c>
-      <c r="D10" s="78" t="s">
+      <c r="D10" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="78" t="s">
+      <c r="B11" s="76" t="s">
         <v>532</v>
       </c>
-      <c r="C11" s="78" t="s">
+      <c r="C11" s="76" t="s">
         <v>366</v>
       </c>
-      <c r="D11" s="78" t="s">
+      <c r="D11" s="76" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="78" t="s">
+      <c r="B12" s="76" t="s">
         <v>533</v>
       </c>
-      <c r="C12" s="78" t="s">
+      <c r="C12" s="76" t="s">
         <v>342</v>
       </c>
-      <c r="D12" s="78" t="s">
+      <c r="D12" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="78" t="s">
+      <c r="B13" s="76" t="s">
         <v>534</v>
       </c>
-      <c r="C13" s="78" t="s">
+      <c r="C13" s="76" t="s">
         <v>366</v>
       </c>
-      <c r="D13" s="78" t="s">
+      <c r="D13" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="78" t="s">
+      <c r="B14" s="76" t="s">
         <v>535</v>
       </c>
-      <c r="C14" s="78" t="s">
+      <c r="C14" s="76" t="s">
         <v>366</v>
       </c>
-      <c r="D14" s="78" t="s">
+      <c r="D14" s="76" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="78" t="s">
+      <c r="B15" s="76" t="s">
         <v>536</v>
       </c>
-      <c r="C15" s="78" t="s">
+      <c r="C15" s="76" t="s">
         <v>342</v>
       </c>
-      <c r="D15" s="78" t="s">
+      <c r="D15" s="76" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B17" s="82"/>
-      <c r="C17" s="82"/>
-      <c r="D17" s="82"/>
-      <c r="E17" s="82"/>
-      <c r="F17" s="82"/>
-      <c r="G17" s="82"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="E17" s="83"/>
+      <c r="F17" s="83"/>
+      <c r="G17" s="83"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B18" s="79" t="s">
+      <c r="B18" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="76" t="s">
         <v>541</v>
       </c>
-      <c r="D18" s="78" t="s">
+      <c r="D18" s="76" t="s">
         <v>542</v>
       </c>
-      <c r="E18" s="78" t="s">
+      <c r="E18" s="76" t="s">
         <v>146</v>
       </c>
-      <c r="F18" s="78" t="s">
+      <c r="F18" s="76" t="s">
         <v>546</v>
       </c>
-      <c r="G18" s="81" t="s">
+      <c r="G18" s="79" t="s">
         <v>548</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B19" s="78" t="s">
+      <c r="B19" s="76" t="s">
         <v>347</v>
       </c>
-      <c r="C19" s="78" t="s">
+      <c r="C19" s="76" t="s">
         <v>347</v>
       </c>
-      <c r="D19" s="78" t="s">
+      <c r="D19" s="76" t="s">
         <v>554</v>
       </c>
-      <c r="E19" s="78" t="s">
+      <c r="E19" s="76" t="s">
         <v>168</v>
       </c>
-      <c r="F19" s="78">
+      <c r="F19" s="76">
         <v>7</v>
       </c>
-      <c r="G19" s="81"/>
+      <c r="G19" s="79"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B20" s="78" t="s">
+      <c r="B20" s="76" t="s">
         <v>385</v>
       </c>
-      <c r="C20" s="78" t="s">
+      <c r="C20" s="76" t="s">
         <v>539</v>
       </c>
-      <c r="D20" s="78" t="s">
+      <c r="D20" s="76" t="s">
         <v>554</v>
       </c>
-      <c r="E20" s="78" t="s">
+      <c r="E20" s="76" t="s">
         <v>168</v>
       </c>
-      <c r="F20" s="78">
+      <c r="F20" s="76">
         <v>8</v>
       </c>
-      <c r="G20" s="78"/>
+      <c r="G20" s="76"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B21" s="78" t="s">
+      <c r="B21" s="76" t="s">
         <v>339</v>
       </c>
-      <c r="C21" s="78" t="s">
+      <c r="C21" s="76" t="s">
         <v>339</v>
       </c>
-      <c r="D21" s="78" t="s">
+      <c r="D21" s="76" t="s">
         <v>554</v>
       </c>
-      <c r="E21" s="78" t="s">
+      <c r="E21" s="76" t="s">
         <v>168</v>
       </c>
-      <c r="F21" s="78">
+      <c r="F21" s="76">
         <v>9</v>
       </c>
-      <c r="G21" s="78"/>
+      <c r="G21" s="76"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B22" s="80"/>
+      <c r="B22" s="78"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B23" s="80"/>
+      <c r="B23" s="78"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B24" s="80"/>
+      <c r="B24" s="78"/>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B25" s="80"/>
+      <c r="B25" s="78"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B26" s="80"/>
+      <c r="B26" s="78"/>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B27" s="80"/>
+      <c r="B27" s="78"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B28" s="80"/>
+      <c r="B28" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9979,4 +10073,320 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDE07AA7-338C-49C8-A26B-C54ECCFE7A1C}">
+  <dimension ref="A1:AJ11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="52.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.5546875" customWidth="1"/>
+    <col min="19" max="19" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="36.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.5546875" customWidth="1"/>
+    <col min="29" max="29" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="5.5546875" customWidth="1"/>
+    <col min="33" max="33" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G1" t="s">
+        <v>556</v>
+      </c>
+      <c r="H1" t="s">
+        <v>146</v>
+      </c>
+      <c r="I1" t="s">
+        <v>218</v>
+      </c>
+      <c r="J1" t="s">
+        <v>146</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
+        <v>146</v>
+      </c>
+      <c r="M1" t="s">
+        <v>90</v>
+      </c>
+      <c r="N1" t="s">
+        <v>146</v>
+      </c>
+      <c r="O1" t="s">
+        <v>560</v>
+      </c>
+      <c r="P1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>576</v>
+      </c>
+      <c r="R1" t="s">
+        <v>146</v>
+      </c>
+      <c r="S1" t="s">
+        <v>14</v>
+      </c>
+      <c r="T1" t="s">
+        <v>146</v>
+      </c>
+      <c r="U1" t="s">
+        <v>12</v>
+      </c>
+      <c r="V1" t="s">
+        <v>146</v>
+      </c>
+      <c r="W1" t="s">
+        <v>563</v>
+      </c>
+      <c r="X1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>223</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>579</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>580</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>570</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>572</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>574</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" t="s">
+        <v>559</v>
+      </c>
+      <c r="F2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" t="s">
+        <v>557</v>
+      </c>
+      <c r="H2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I2" t="s">
+        <v>218</v>
+      </c>
+      <c r="J2" t="s">
+        <v>185</v>
+      </c>
+      <c r="K2" t="s">
+        <v>91</v>
+      </c>
+      <c r="L2" t="s">
+        <v>160</v>
+      </c>
+      <c r="M2" t="s">
+        <v>90</v>
+      </c>
+      <c r="N2" t="s">
+        <v>155</v>
+      </c>
+      <c r="O2" t="s">
+        <v>119</v>
+      </c>
+      <c r="P2" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>577</v>
+      </c>
+      <c r="R2" t="s">
+        <v>220</v>
+      </c>
+      <c r="S2" t="s">
+        <v>561</v>
+      </c>
+      <c r="T2" t="s">
+        <v>290</v>
+      </c>
+      <c r="U2" t="s">
+        <v>12</v>
+      </c>
+      <c r="V2" t="s">
+        <v>562</v>
+      </c>
+      <c r="W2" t="s">
+        <v>563</v>
+      </c>
+      <c r="X2" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>564</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>209</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>578</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>504</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>580</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>213</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>570</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>571</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>572</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>573</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>575</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A7" s="84" t="s">
+        <v>569</v>
+      </c>
+      <c r="B7" s="84"/>
+      <c r="C7" s="84"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A8" s="76" t="s">
+        <v>568</v>
+      </c>
+      <c r="B8" s="76" t="s">
+        <v>567</v>
+      </c>
+      <c r="C8" s="76" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A9" s="76" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="76" t="s">
+        <v>565</v>
+      </c>
+      <c r="C9" s="76" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A10" s="76" t="s">
+        <v>218</v>
+      </c>
+      <c r="B10" s="76" t="s">
+        <v>374</v>
+      </c>
+      <c r="C10" s="76" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A11" s="76" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="76" t="s">
+        <v>349</v>
+      </c>
+      <c r="C11" s="76" t="s">
+        <v>342</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A7:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>